<commit_message>
Se hizo cambios en extraer_carpeta.py y visor_planos.html... para que reconociera solo las piezas 090 que estan en las carpetas
</commit_message>
<xml_diff>
--- a/output/DWG_planos.xlsx
+++ b/output/DWG_planos.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Raiz" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="pieza 90" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -577,4 +578,186 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Archivo</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Tabla</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Campo</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Valor</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>423 07 090.dwg</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>BN+D</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>BN+D</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>423 07 090.dwg</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>OFFSET</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>423 07 090.dwg</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>BN+D</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>40+5</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>423 07 090.dwg</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>3</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>OFFSET</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>423 07 090.dwg</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>3</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>BN+D</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>38+5</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>423 07 090.dwg</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>4</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>OFFSET</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>423 07 090.dwg</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>4</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>BN+D</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>40+5</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
se corigio el bug de las tablas con los mismos nombres... si varias tablas tenian en BN+D = 91 y otra tabla con el mismo BN+D = 96+5, ahora si coge las dos tablas porque antes solo codiga una...
</commit_message>
<xml_diff>
--- a/output/DWG_planos.xlsx
+++ b/output/DWG_planos.xlsx
@@ -8,7 +8,9 @@
   </bookViews>
   <sheets>
     <sheet name="Raiz" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="pieza 90" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="V-05 BLINTECH" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="V-05 BLINTECH_PLANOS DE APROBAC" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="pieza 90" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -586,6 +588,330 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Archivo</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Tabla</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Campo</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Valor</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>logan pruena 006 090.dwg</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>OFFSET</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>logan pruena 006 090.dwg</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>BN+D</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>79+5</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>logan pruena 006 090.dwg</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>OFFSET</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>logan pruena 006 090.dwg</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>BN+D</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>108+5</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>logan pruena 006 090.dwg</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>3</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>OFFSET</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>logan pruena 006 090.dwg</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>3</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>BN+D</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>80+5</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Archivo</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Tabla</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Campo</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Valor</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>LOGAN DOS 006 090.dwg</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>OFFSET</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>LOGAN DOS 006 090.dwg</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>BN+D</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>79+5</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>LOGAN DOS 006 090.dwg</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>OFFSET</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>LOGAN DOS 006 090.dwg</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>BN+D</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>108+5</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>LOGAN DOS 006 090.dwg</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>3</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>OFFSET</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>LOGAN DOS 006 090.dwg</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>3</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>BN+D</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>80+5</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>